<commit_message>
Complete export center integration
</commit_message>
<xml_diff>
--- a/Backend/exports/test_cases.xlsx
+++ b/Backend/exports/test_cases.xlsx
@@ -446,12 +446,16 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify Login</t>
+          <t>Verify Login Test
+1. Open login page
+2. Enter credentials
+3. Click login
+4. Verify dashboard</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>POS</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>